<commit_message>
Corrida | SFE-ESCT | 2026-06-17 11:33:10.577709
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ESCT_out.xlsx
+++ b/indicadores/SFE-ESCT_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="417">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Escrituras de ventas en la provincia de Santa Fe</t>
+    <t xml:space="preserve">Escrituras de ventas</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">20/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1761,9 +1767,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1774,7 +1784,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1788,12 +1798,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.361841837594438</v>
+        <v>0.366124166029138</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1804,7 +1814,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1832,7 +1842,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1846,12 +1856,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.13092951543372</v>
+        <v>0.134046904950532</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1874,7 +1884,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1888,7 +1898,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1902,7 +1912,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1916,12 +1926,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00629848998263466</v>
+        <v>0.00744822137426289</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1932,7 +1942,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1946,12 +1956,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0000222215316886116</v>
+        <v>0.0000299063199286307</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2094,10 +2104,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2110,10 +2120,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2137,66 +2147,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>2450</v>
@@ -2249,7 +2259,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>2775</v>
@@ -2306,7 +2316,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>3696</v>
@@ -2363,7 +2373,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>3429</v>
@@ -2420,7 +2430,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>2099</v>
@@ -2477,7 +2487,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>3249</v>
@@ -2534,7 +2544,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>4020</v>
@@ -2591,7 +2601,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>3331</v>
@@ -2648,7 +2658,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>3288</v>
@@ -2705,7 +2715,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>2883</v>
@@ -2762,7 +2772,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>3607</v>
@@ -2819,7 +2829,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>4078</v>
@@ -2876,7 +2886,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>2012</v>
@@ -2935,7 +2945,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>2347</v>
@@ -2994,7 +3004,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>3083</v>
@@ -3053,7 +3063,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>3260</v>
@@ -3112,7 +3122,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>3356</v>
@@ -3171,7 +3181,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>3333</v>
@@ -3230,7 +3240,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>3387</v>
@@ -3289,7 +3299,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>3488</v>
@@ -3348,7 +3358,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>3735</v>
@@ -3407,7 +3417,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>3318</v>
@@ -3466,7 +3476,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>3198</v>
@@ -3525,7 +3535,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>4248</v>
@@ -3584,7 +3594,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>2205</v>
@@ -3643,7 +3653,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>2480</v>
@@ -3702,7 +3712,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>3358</v>
@@ -3761,7 +3771,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>3198</v>
@@ -3820,7 +3830,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>3385</v>
@@ -3879,7 +3889,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>3668</v>
@@ -3938,7 +3948,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>3263</v>
@@ -3997,7 +4007,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>3835</v>
@@ -4056,7 +4066,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>3658</v>
@@ -4115,7 +4125,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>3770</v>
@@ -4174,7 +4184,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>3396</v>
@@ -4233,7 +4243,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>3917</v>
@@ -4292,7 +4302,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>2401</v>
@@ -4351,7 +4361,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>3413</v>
@@ -4410,7 +4420,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>4205</v>
@@ -4469,7 +4479,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>2760</v>
@@ -4528,7 +4538,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>2702</v>
@@ -4587,7 +4597,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>3916</v>
@@ -4646,7 +4656,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>3365</v>
@@ -4705,7 +4715,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>4022</v>
@@ -4764,7 +4774,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>3739</v>
@@ -4823,7 +4833,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>3590</v>
@@ -4882,7 +4892,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>3083</v>
@@ -4941,7 +4951,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>5506</v>
@@ -5000,7 +5010,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>2039</v>
@@ -5059,7 +5069,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>2753</v>
@@ -5118,7 +5128,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>3251</v>
@@ -5177,7 +5187,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>3496</v>
@@ -5236,7 +5246,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>3915</v>
@@ -5295,7 +5305,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>3483</v>
@@ -5354,7 +5364,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>3738</v>
@@ -5413,7 +5423,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>3236</v>
@@ -5472,7 +5482,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>3309</v>
@@ -5531,7 +5541,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>3399</v>
@@ -5590,7 +5600,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>3415</v>
@@ -5649,7 +5659,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>3711</v>
@@ -5708,7 +5718,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>1450</v>
@@ -5767,7 +5777,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>1975</v>
@@ -5826,7 +5836,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>2671</v>
@@ -5885,7 +5895,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>2466</v>
@@ -5944,7 +5954,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>2500</v>
@@ -6003,7 +6013,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>2705</v>
@@ -6062,7 +6072,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>2731</v>
@@ -6121,7 +6131,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>2746</v>
@@ -6180,7 +6190,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>2934</v>
@@ -6239,7 +6249,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>2956</v>
@@ -6298,7 +6308,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>2862</v>
@@ -6357,7 +6367,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>3732</v>
@@ -6416,7 +6426,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>1668</v>
@@ -6475,7 +6485,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>2036</v>
@@ -6534,7 +6544,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>2138</v>
@@ -6593,7 +6603,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>3372</v>
@@ -6652,7 +6662,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>3021</v>
@@ -6711,7 +6721,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>2939</v>
@@ -6770,7 +6780,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>3612</v>
@@ -6829,7 +6839,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>2864</v>
@@ -6888,7 +6898,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>3322</v>
@@ -6947,7 +6957,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>3122</v>
@@ -7006,7 +7016,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>3759</v>
@@ -7065,7 +7075,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>4226</v>
@@ -7124,7 +7134,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>1961</v>
@@ -7183,7 +7193,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>2242</v>
@@ -7242,7 +7252,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>2729</v>
@@ -7301,7 +7311,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>3680</v>
@@ -7360,7 +7370,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>3604</v>
@@ -7419,7 +7429,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>3740</v>
@@ -7478,7 +7488,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>4791</v>
@@ -7537,7 +7547,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>4042</v>
@@ -7596,7 +7606,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>3772</v>
@@ -7655,7 +7665,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>3499</v>
@@ -7714,7 +7724,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>3820</v>
@@ -7773,7 +7783,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>4607</v>
@@ -7832,7 +7842,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>2171</v>
@@ -7891,7 +7901,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>2172</v>
@@ -7950,7 +7960,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>3341</v>
@@ -8009,7 +8019,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>2790</v>
@@ -8068,7 +8078,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>3385</v>
@@ -8127,7 +8137,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>3269</v>
@@ -8186,7 +8196,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>3196</v>
@@ -8245,7 +8255,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>3551</v>
@@ -8304,7 +8314,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>3052</v>
@@ -8363,7 +8373,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>2991</v>
@@ -8422,7 +8432,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>3177</v>
@@ -8481,7 +8491,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>3495</v>
@@ -8540,7 +8550,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>1781</v>
@@ -8599,7 +8609,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>1851</v>
@@ -8658,7 +8668,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>3094</v>
@@ -8717,7 +8727,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>2712</v>
@@ -8776,7 +8786,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>3527</v>
@@ -8835,7 +8845,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>3091</v>
@@ -8894,7 +8904,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>3172</v>
@@ -8953,7 +8963,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>3321</v>
@@ -9012,7 +9022,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>3216</v>
@@ -9071,7 +9081,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>3345</v>
@@ -9130,7 +9140,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>3222</v>
@@ -9189,7 +9199,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>3821</v>
@@ -9248,7 +9258,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>2508</v>
@@ -9307,7 +9317,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>2149</v>
@@ -9366,7 +9376,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>2631</v>
@@ -9425,7 +9435,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>2799</v>
@@ -9484,7 +9494,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>2539</v>
@@ -9543,7 +9553,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>2795</v>
@@ -9602,7 +9612,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>3338</v>
@@ -9661,7 +9671,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>3118</v>
@@ -9720,7 +9730,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>2955</v>
@@ -9779,7 +9789,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>3319</v>
@@ -9838,7 +9848,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>2800</v>
@@ -9897,7 +9907,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>3086</v>
@@ -9956,7 +9966,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>2091</v>
@@ -10015,7 +10025,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>1863</v>
@@ -10074,7 +10084,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>2242</v>
@@ -10133,7 +10143,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>2552</v>
@@ -10192,7 +10202,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>2625</v>
@@ -10251,7 +10261,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>2633</v>
@@ -10310,7 +10320,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>2638</v>
@@ -10369,7 +10379,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>2658</v>
@@ -10428,7 +10438,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>2701</v>
@@ -10487,7 +10497,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>2484</v>
@@ -10546,7 +10556,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>2869</v>
@@ -10605,7 +10615,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>2837</v>
@@ -10664,7 +10674,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>1577</v>
@@ -10723,7 +10733,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>1532</v>
@@ -10782,7 +10792,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>2164</v>
@@ -10841,7 +10851,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>2239</v>
@@ -10900,7 +10910,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>2177</v>
@@ -10959,7 +10969,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>2184</v>
@@ -11018,7 +11028,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>1810</v>
@@ -11077,7 +11087,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>2351</v>
@@ -11136,7 +11146,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>2443</v>
@@ -11195,7 +11205,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>2471</v>
@@ -11254,7 +11264,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>2468</v>
@@ -11313,7 +11323,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>2795</v>
@@ -11372,7 +11382,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>1905</v>
@@ -11431,7 +11441,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>1666</v>
@@ -11490,7 +11500,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>2303</v>
@@ -11549,7 +11559,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>2000</v>
@@ -11608,7 +11618,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>2437</v>
@@ -11667,7 +11677,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>2912</v>
@@ -11726,7 +11736,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>2543</v>
@@ -11785,7 +11795,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>2208</v>
@@ -11844,7 +11854,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>3100</v>
@@ -11903,7 +11913,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>2714</v>
@@ -11962,7 +11972,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>3195</v>
@@ -12021,7 +12031,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>3129</v>
@@ -12080,7 +12090,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>2170</v>
@@ -12139,7 +12149,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>2107</v>
@@ -12198,7 +12208,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>2723</v>
@@ -12257,7 +12267,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>2883</v>
@@ -12316,7 +12326,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>2971</v>
@@ -12375,7 +12385,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>3098</v>
@@ -12434,7 +12444,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>2338</v>
@@ -12493,7 +12503,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>2468</v>
@@ -12552,7 +12562,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>2213</v>
@@ -12611,7 +12621,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>2149</v>
@@ -12670,7 +12680,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>2622</v>
@@ -12729,7 +12739,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>2676</v>
@@ -12788,7 +12798,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>1715</v>
@@ -12847,7 +12857,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>1575</v>
@@ -12906,7 +12916,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>1900</v>
@@ -12965,7 +12975,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>2283</v>
@@ -13024,7 +13034,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>2237</v>
@@ -13083,7 +13093,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>2181</v>
@@ -13142,7 +13152,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>1936</v>
@@ -13201,7 +13211,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>2223</v>
@@ -13260,7 +13270,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>2068</v>
@@ -13319,7 +13329,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>1901</v>
@@ -13378,7 +13388,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>1699</v>
@@ -13437,7 +13447,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>2267</v>
@@ -13496,7 +13506,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>1668</v>
@@ -13555,7 +13565,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>1482</v>
@@ -13614,7 +13624,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>1448</v>
@@ -13673,7 +13683,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>218</v>
@@ -13732,7 +13742,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>550</v>
@@ -13791,7 +13801,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>1391</v>
@@ -13850,7 +13860,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>1882</v>
@@ -13909,7 +13919,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>2291</v>
@@ -13968,7 +13978,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>2370</v>
@@ -14027,7 +14037,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>1974</v>
@@ -14086,7 +14096,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>2562</v>
@@ -14145,7 +14155,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>2762</v>
@@ -14204,7 +14214,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>2111</v>
@@ -14263,7 +14273,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>1838</v>
@@ -14322,7 +14332,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>2903</v>
@@ -14381,7 +14391,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>2509</v>
@@ -14440,7 +14450,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>1810</v>
@@ -14499,7 +14509,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>2016</v>
@@ -14558,7 +14568,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>2760</v>
@@ -14617,7 +14627,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>2581</v>
@@ -14676,7 +14686,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>2680</v>
@@ -14735,7 +14745,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>2580</v>
@@ -14794,7 +14804,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>2658</v>
@@ -14853,7 +14863,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>2313</v>
@@ -14912,7 +14922,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>1700</v>
@@ -14971,7 +14981,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>1659</v>
@@ -15030,7 +15040,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>2276</v>
@@ -15089,7 +15099,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>2531</v>
@@ -15148,7 +15158,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>2256</v>
@@ -15207,7 +15217,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>2223</v>
@@ -15266,7 +15276,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>2417</v>
@@ -15325,7 +15335,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>2341</v>
@@ -15384,7 +15394,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>2394</v>
@@ -15443,7 +15453,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>2562</v>
@@ -15502,7 +15512,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>2519</v>
@@ -15561,7 +15571,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>2623</v>
@@ -15620,7 +15630,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>1813</v>
@@ -15679,7 +15689,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>1641</v>
@@ -15738,7 +15748,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>1983</v>
@@ -15797,7 +15807,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>2253</v>
@@ -15856,7 +15866,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>1875</v>
@@ -15915,7 +15925,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>2068</v>
@@ -15974,7 +15984,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>2007</v>
@@ -16033,7 +16043,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>2275</v>
@@ -16092,7 +16102,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>2423</v>
@@ -16151,7 +16161,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>2396</v>
@@ -16210,7 +16220,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>1866</v>
@@ -16269,7 +16279,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>2404</v>
@@ -16328,7 +16338,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>1556</v>
@@ -16387,7 +16397,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>1408</v>
@@ -16446,7 +16456,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>763</v>
@@ -16505,7 +16515,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>1619</v>
@@ -16564,7 +16574,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>2212</v>
@@ -16623,7 +16633,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>2613</v>
@@ -16682,7 +16692,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>2133</v>
@@ -16741,7 +16751,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>2712</v>
@@ -16800,7 +16810,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>2519</v>
@@ -16859,7 +16869,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>3096</v>
@@ -16918,7 +16928,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>2472</v>
@@ -16977,7 +16987,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>2918</v>
@@ -17036,7 +17046,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>2405</v>
@@ -17095,7 +17105,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>2574</v>
@@ -17154,7 +17164,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>2632</v>
@@ -17213,7 +17223,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>2914</v>
@@ -17272,7 +17282,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>2770</v>
@@ -17331,7 +17341,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>4060</v>
@@ -17390,7 +17400,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>3501</v>
@@ -17449,7 +17459,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>3169</v>
@@ -17508,7 +17518,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>3348</v>
@@ -17567,7 +17577,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>3477</v>
@@ -17626,7 +17636,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>3035</v>
@@ -17685,7 +17695,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>3709</v>
@@ -17744,7 +17754,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>2034</v>
@@ -17803,7 +17813,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>2223</v>
@@ -17862,7 +17872,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>3185</v>
@@ -17921,7 +17931,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B269" s="2"/>
       <c r="C269" s="3" t="n">
@@ -17954,7 +17964,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B270" s="2"/>
       <c r="C270" s="3" t="n">
@@ -17987,7 +17997,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B271" s="2"/>
       <c r="C271" s="3" t="n">
@@ -18020,7 +18030,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B272" s="2"/>
       <c r="C272" s="3" t="n">
@@ -18053,7 +18063,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B273" s="2"/>
       <c r="C273" s="3" t="n">
@@ -18086,7 +18096,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B274" s="2"/>
       <c r="C274" s="3" t="n">
@@ -18119,7 +18129,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B275" s="2"/>
       <c r="C275" s="3" t="n">
@@ -18152,7 +18162,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B276" s="2"/>
       <c r="C276" s="3" t="n">
@@ -18185,7 +18195,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B277" s="2"/>
       <c r="C277" s="3" t="n">
@@ -18218,7 +18228,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B278" s="2"/>
       <c r="C278" s="3" t="n">
@@ -18251,7 +18261,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B279" s="2"/>
       <c r="C279" s="3" t="n">
@@ -18284,7 +18294,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B280" s="2"/>
       <c r="C280" s="3" t="n">
@@ -18317,7 +18327,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B281" s="2"/>
       <c r="C281" s="3"/>
@@ -18340,7 +18350,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B282" s="2"/>
       <c r="C282" s="3"/>
@@ -18363,7 +18373,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B283" s="2"/>
       <c r="C283" s="3"/>
@@ -18386,7 +18396,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B284" s="2"/>
       <c r="C284" s="3"/>
@@ -18409,7 +18419,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B285" s="2"/>
       <c r="C285" s="3"/>
@@ -18432,7 +18442,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B286" s="2"/>
       <c r="C286" s="3"/>
@@ -18455,7 +18465,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B287" s="2"/>
       <c r="C287" s="3"/>
@@ -18478,7 +18488,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B288" s="2"/>
       <c r="C288" s="3"/>
@@ -18501,7 +18511,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B289" s="2"/>
       <c r="C289" s="3"/>
@@ -18524,7 +18534,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B290" s="2"/>
       <c r="C290" s="3"/>
@@ -18547,7 +18557,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B291" s="2"/>
       <c r="C291" s="3"/>
@@ -18570,7 +18580,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B292" s="2"/>
       <c r="C292" s="3"/>
@@ -18593,7 +18603,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B293" s="2"/>
       <c r="C293" s="3"/>
@@ -18616,7 +18626,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B294" s="2"/>
       <c r="C294" s="3"/>
@@ -18639,7 +18649,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B295" s="2"/>
       <c r="C295" s="3"/>
@@ -18662,7 +18672,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B296" s="2"/>
       <c r="C296" s="3"/>
@@ -18685,7 +18695,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B297" s="2"/>
       <c r="C297" s="3"/>
@@ -18708,7 +18718,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B298" s="2"/>
       <c r="C298" s="3"/>
@@ -18731,7 +18741,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B299" s="2"/>
       <c r="C299" s="3"/>
@@ -18754,7 +18764,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B300" s="2"/>
       <c r="C300" s="3"/>
@@ -18777,7 +18787,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B301" s="2"/>
       <c r="C301" s="3"/>
@@ -18800,7 +18810,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B302" s="2"/>
       <c r="C302" s="3"/>
@@ -18823,7 +18833,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B303" s="2"/>
       <c r="C303" s="3"/>
@@ -18846,7 +18856,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B304" s="2"/>
       <c r="C304" s="3"/>
@@ -18869,7 +18879,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B305" s="2"/>
       <c r="C305" s="3"/>
@@ -18892,7 +18902,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B306" s="2"/>
       <c r="C306" s="3"/>
@@ -18915,7 +18925,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B307" s="2"/>
       <c r="C307" s="3"/>
@@ -18938,7 +18948,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B308" s="2"/>
       <c r="C308" s="3"/>
@@ -18961,7 +18971,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B309" s="2"/>
       <c r="C309" s="3"/>
@@ -18984,7 +18994,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B310" s="2"/>
       <c r="C310" s="3"/>
@@ -19007,7 +19017,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B311" s="2"/>
       <c r="C311" s="3"/>
@@ -19030,7 +19040,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B312" s="2"/>
       <c r="C312" s="3"/>
@@ -19053,7 +19063,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B313" s="2"/>
       <c r="C313" s="3"/>
@@ -19076,7 +19086,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B314" s="2"/>
       <c r="C314" s="3"/>
@@ -19099,7 +19109,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B315" s="2"/>
       <c r="C315" s="3"/>
@@ -19122,7 +19132,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B316" s="2"/>
       <c r="C316" s="3"/>
@@ -19145,7 +19155,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B317" s="2"/>
       <c r="C317" s="3"/>
@@ -19168,7 +19178,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B318" s="2"/>
       <c r="C318" s="3"/>
@@ -19191,7 +19201,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B319" s="2"/>
       <c r="C319" s="3"/>
@@ -19214,7 +19224,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B320" s="2"/>
       <c r="C320" s="3"/>
@@ -19237,7 +19247,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B321" s="2"/>
       <c r="C321" s="3"/>
@@ -19260,7 +19270,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B322" s="2"/>
       <c r="C322" s="3"/>
@@ -19283,7 +19293,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B323" s="2"/>
       <c r="C323" s="3"/>
@@ -19306,7 +19316,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B324" s="2"/>
       <c r="C324" s="3"/>
@@ -19329,7 +19339,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B325" s="2"/>
       <c r="C325" s="3"/>
@@ -19363,97 +19373,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
   </sheetData>
@@ -19477,7 +19487,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -19487,160 +19497,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0160903792380331</v>
+        <v>-0.0158495534531084</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0454155320925058</v>
+        <v>0.0442048119641213</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0804997562930156</v>
+        <v>0.0790403333245629</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0966913415462876</v>
+        <v>0.0948386108170693</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.0642070524969603</v>
+        <v>0.0646384495579988</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.136782000288217</v>
+        <v>0.13785791379015</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.287900362391146</v>
+        <v>0.286075722286673</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.330603790177407</v>
+        <v>0.328726901758079</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.345380554076528</v>
+        <v>0.3476562131465</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.361841837594438</v>
+        <v>0.366124166029138</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.325298499893017</v>
+        <v>0.32697276568767</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.275153658018249</v>
+        <v>0.274424325709588</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.194691598900623</v>
+        <v>0.194057420267942</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.137844811883563</v>
+        <v>0.138572142791302</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.132522233177547</v>
+        <v>0.133705600307888</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0552516418075085</v>
+        <v>0.0568430708211685</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0460252792787931</v>
+        <v>-0.0436180540647462</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.11439132024549</v>
+        <v>-0.112127747848774</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.202827851512636</v>
+        <v>-0.200716240140229</v>
       </c>
     </row>
     <row r="24">

</xml_diff>